<commit_message>
TENDERS_1210.xlsx: add unit prices per position and average unit price; med and cable lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TENDERS_1210.xlsx
+++ b/TENDERS_1210.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$N$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$P$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,16 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -73,15 +83,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -448,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -458,13 +473,15 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,35 +522,45 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Позиции: кол-во × цена за ед. в НМЦК, ₽</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Средняя цена за ед. в НМЦК, ₽</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Себестоимость, ₽</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Валовая маржа при НМЦК</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ожид. снижение</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Прибыль при НМЦК, ₽</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Прибыль при ожид. снижении, ₽</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Решение</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -557,7 +584,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Соль техническая 948 т (14 630 ₽/т)</t>
+          <t>Соль техническая 948 т</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -573,27 +600,35 @@
       <c r="G2" s="2" t="n">
         <v>13869240</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>948 т × 14 630 ₽/т</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>14630</v>
+      </c>
+      <c r="J2" s="2" t="n">
         <v>2370000</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="K2" s="4" t="n">
         <v>0.8291182501708817</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="L2" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="M2" s="2" t="n">
         <v>9262976.735973697</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>7859631.555813699</v>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Участвовать</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ на эквивалент</t>
         </is>
@@ -617,7 +652,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Соль техническая 400 т (16 810 ₽/т)</t>
+          <t>Соль техническая 400 т</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -633,27 +668,35 @@
       <c r="G3" s="2" t="n">
         <v>6724000</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>400 т × 16 810 ₽/т</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>16810</v>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="K3" s="4" t="n">
         <v>0.851279000594884</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="L3" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>4621641.290520548</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>3941280.074520547</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Участвовать</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>223-ФЗ; обеспечение исполнения 10%</t>
         </is>
@@ -677,7 +720,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Соль техническая 130 т (12 260 ₽/т)</t>
+          <t>Соль техническая 130 т</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -693,27 +736,35 @@
       <c r="G4" s="2" t="n">
         <v>1593800</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>130 т × 12 260 ₽/т</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>12260</v>
+      </c>
+      <c r="J4" s="2" t="n">
         <v>325000</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="K4" s="4" t="n">
         <v>0.7960848287112561</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="L4" s="4" t="n">
         <v>0.03</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="M4" s="2" t="n">
         <v>1018243.203419178</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>856976.144219178</v>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Участвовать</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ</t>
         </is>
@@ -722,22 +773,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Одежда</t>
+          <t>Медрасходники</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0372100027326000601</t>
+          <t>0373200001326001396</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Федеральное бюджетное учреждение «Администрация Волго-Балтийского бассейна внутренних водных путей»</t>
+          <t>ГБУЗ г. Москвы «ГКБ им. В.В. Вересаева ДЗМ»</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Поставка средств индивидуальной защиты, приобретаемых для нужд ФБУ «Администрация «Волго-Балт» (44-ФЗ)</t>
+          <t>Пробирки вакуумные с активатором</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -747,95 +798,111 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-13 10:00</t>
+          <t>15.10.2026 09:00 МСК</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>18033874.9</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>13525406.175</v>
-      </c>
-      <c r="I5" s="3" t="n">
+        <v>2952000</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с активатором свертывания,: 150 000 шт × 19.68</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>19.68</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1446500</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.5099932249322493</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J5" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>2571289.646392574</v>
-      </c>
-      <c r="L5" s="2" t="n">
-        <v>2571289.646392574</v>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>Участвовать, если ≤2 заявок</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
+      <c r="M5" s="2" t="n">
+        <v>1178755.920547945</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>556474.3205479452</v>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Участвовать</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>НМЦК 19,68 ₽ — вдвое выше рынка, поэтому ожидается сильное снижение (вероятно верхний квартиль скидки, 40–55%). Особенность крышки (полнозаходная резьба / двухступенчатое снятие) — нужно подтвердить, что UNIVAC/другая российская пробирка этому соответствует, иначе отклонение. СМП-only. Минимальный о</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Одежда</t>
+          <t>Кабель (ЭОМ)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0358200022926000030</t>
+          <t>32616447145</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ГКУ Ростовской обл. «Ростовская областная поисково-спасательная служба»</t>
+          <t>АО «Пассажирречтранс»</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Поставка обмундирования</t>
+          <t>Кабель (27.32)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-19 09:00</t>
+          <t>16.10.2026 05:00 МСК (09:00 местн.)</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>6224420.7</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>4668315.525</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>887484.7246889586</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>887484.7246889586</v>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Участвовать, если ≤2 заявок</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
+        <v>450798.91</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Кабель судовой КНР и КНРЭ (ГОСТ 7866.1-76), с: 1 730 м × 260.58</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>260.5774046242774</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>281420</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.3757305225072527</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>136974.4710489863</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>68554.01568482628</v>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Участвовать</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Сечения и доля КНРЭ неизвестны — себестоимость гипотетична. Розничные цены агрегаторов (Рукабель, kabel-s) 170–440 ₽/м выше средней НМЦК 260,6 ₽/м → если в лоте 3х2,5 и крупнее, маржи может не быть; реально только при цене завода (Кольчугино/Рыбинсккабель/Камкабель) ~126–154 ₽/м за 3х2,5 и малых сеч</t>
         </is>
       </c>
     </row>
@@ -847,53 +914,63 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>32616443256</t>
+          <t>0372100027326000601</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ГБУ Республики Саха (Якутия) «Государственная Противопожарная Служба Республики Саха(Якутия)»</t>
+          <t>Федеральное бюджетное учреждение «Администрация Волго-Балтийского бассейна внутренних водных путей»</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Поставка форменной одежды для нужд ГБУ РС(Я) "ГПС РС(Я)"</t>
+          <t>Поставка средств индивидуальной защиты, приобретаемых для нужд ФБУ «Администрация «Волго-Балт» (44-ФЗ)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>223-ФЗ</t>
+          <t>44-ФЗ</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-15 05:00</t>
+          <t>2026-10-13 10:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>4999001.85</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>3749251.3875</v>
-      </c>
-      <c r="I7" s="3" t="n">
+        <v>18033874.9</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Костюм для защиты от термических рисков элект: 1 КОМПЛ × 4 865.60; Строп одинарный регулируемый огнеупорный: 4 шт × 2 379.09; Каска защитная белая: 31 шт × 551.06; Гибкая анкерная линия (20 м): 2 шт × 2 765.56; Наколенники: 15 пар × 871.08; Белье нательное термостойкое: 192 КОМПЛ × 1 741.12; Одежда специальная повышенной видимости: 18 шт × 142.69; Обувь специальная кожаная для защиты от механ: 72 пар × 2 125.85; … ещё 126</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>разные позиции — см. колонку слева</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>13525406.175</v>
+      </c>
+      <c r="K7" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="L7" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K7" s="2" t="n">
-        <v>712763.1621311915</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>712763.1621311915</v>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="M7" s="2" t="n">
+        <v>2571289.646392574</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>2571289.646392574</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -907,53 +984,63 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32616438570</t>
+          <t>0358200022926000030</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ООО «Теплоэнергетическая Компания - 2»</t>
+          <t>ГКУ Ростовской обл. «Ростовская областная поисково-спасательная служба»</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Поставка зимней спецодежды</t>
+          <t>Поставка обмундирования</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>223-ФЗ</t>
+          <t>44-ФЗ</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-14 08:00</t>
+          <t>2026-10-19 09:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>4810413.58</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>3607810.185</v>
-      </c>
-      <c r="I8" s="3" t="n">
+        <v>6224420.7</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Костюм спасателя зимний (куртка, брюки утепле: 168 КОМПЛ × 7 698.83; Костюм спасателя летний (куртка, брюки, кепка: 241 КОМПЛ × 6 613.44; Комбинезон спасателя зимний, шт.: 208 шт × 7 565.57; Комбинезон спасателя летний, шт.: 239 шт × 6 542.14; Футболка форменная, шт.: 268 шт × 746.15</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>разные позиции — см. колонку слева</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>4668315.525</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="L8" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K8" s="2" t="n">
-        <v>685874.0399225147</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>685874.0399225147</v>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="2" t="n">
+        <v>887484.7246889586</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>887484.7246889586</v>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -967,53 +1054,61 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ГП622514</t>
+          <t>32616443256</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>АО «Арго»</t>
+          <t>ГБУ Республики Саха (Якутия) «Государственная Противопожарная Служба Республики Саха(Якутия)»</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Закупка спецодежды, обуви и средств индивидуальной защиты</t>
+          <t>Поставка форменной одежды для нужд ГБУ РС(Я) "ГПС РС(Я)"</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Коммерческие</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-15 17:00</t>
+          <t>2026-10-15 05:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="I9" s="3" t="n">
+        <v>4999001.85</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Костюм летний полевой: 405 Комплект × ?; Зимняя форменная одежда мужская: 150 Комплект × ? (цена за ед. = НМЦК / кол-во)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>9007.21054054054</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>3749251.3875</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="L9" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K9" s="2" t="n">
-        <v>570324.3835616438</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>570324.3835616438</v>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="2" t="n">
+        <v>712763.1621311915</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>712763.1621311915</v>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1027,17 +1122,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>32616402062</t>
+          <t>32616438570</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>МУП «Управление Городского Хозяйства» Муниципального Образования Города Пыть-Ях</t>
+          <t>ООО «Теплоэнергетическая Компания - 2»</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Поставка специальных обуви, одежды, головных уборов, рукавиц и краг</t>
+          <t>Поставка зимней спецодежды</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1047,33 +1142,41 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-10-13 06:00</t>
+          <t>2026-10-14 08:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>3857857.45</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>2893393.0875</v>
-      </c>
-      <c r="I10" s="3" t="n">
+        <v>4810413.58</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Костюм мужской для защиты от пониженных темпе: 391 Штука × ?; Костюм сварщика со спилком утепленный: 20 Штука × ?; Костюм женский утепленный: 41 Штука × ?; Костюм зимний мужской для защиты от термическ: 28 Штука × ?; Куртка охранника зимняя: 46 Штука × ?; Брюки охранника зимние: 46 Штука × ?; Шеврон на липучке для спецодежды: 46 Штука × ?; Костюм мужской для защиты от пониженных темпе: 391 Штука × ?; … ещё 6 (цена за ед. = НМЦК / кол-во)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>3891.920372168285</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>3607810.185</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="L10" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K10" s="2" t="n">
-        <v>550057.5430099862</v>
-      </c>
-      <c r="L10" s="2" t="n">
-        <v>550057.5430099862</v>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="2" t="n">
+        <v>685874.0399225147</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>685874.0399225147</v>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1087,53 +1190,59 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>32616431081</t>
+          <t>ГП622514</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Федеральное бюджетное учреждение «Государственный Региональный Центр Стандартизации, Метрологии и Испытаний Им. А.М. Муратшина в Республике Башкортостан»</t>
+          <t>АО «Арго»</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Поставка спецодежды</t>
+          <t>Закупка спецодежды, обуви и средств индивидуальной защиты</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>223-ФЗ</t>
+          <t>Коммерческие</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-19 08:00</t>
+          <t>2026-10-15 17:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>3637476.36</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>2728107.27</v>
-      </c>
-      <c r="I11" s="3" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="K11" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="L11" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K11" s="2" t="n">
-        <v>518635.365684263</v>
-      </c>
-      <c r="L11" s="2" t="n">
-        <v>518635.365684263</v>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="2" t="n">
+        <v>570324.3835616438</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>570324.3835616438</v>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1147,17 +1256,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>32616448893</t>
+          <t>32616402062</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Государственное автономное учреждение Московской обл. «Мособллес»</t>
+          <t>МУП «Управление Городского Хозяйства» Муниципального Образования Города Пыть-Ях</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Поставка обуви специальной для защиты от механических воздействий</t>
+          <t>Поставка специальных обуви, одежды, головных уборов, рукавиц и краг</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1167,33 +1276,43 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-10-16 10:00</t>
+          <t>2026-10-13 06:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>2511958.68</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>1883969.01</v>
-      </c>
-      <c r="I12" s="3" t="n">
+        <v>3857857.45</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Ботинки кожаные утепленные: 46 Пара (2 шт.) × ?; Сапоги кожаные утепленные: 185 Пара (2 шт.) × ?; Сапоги утепленные "Надым" ТХ-011р/п с КП и АС: 21 Пара (2 шт.) × ?; Валенки с резиновым низом: 40 Пара (2 шт.) × ?; Костюм сварщика утепленный (4 класс защиты): 8 Штука × ?; Костюм от пониженных температур (4 класс защи: 115 Штука × ?; Костюм сигнальный с водоотталкивающей пропитк: 41 Штука × ?; Костюм зимний петролеум плюс куртка-П/К, Т.Си: 21 Штука × ?; … ещё 18</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>2893393.0875</v>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="L12" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K12" s="2" t="n">
-        <v>358157.8214258302</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>358157.8214258302</v>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="2" t="n">
+        <v>550057.5430099862</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>550057.5430099862</v>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1207,7 +1326,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>32616427138</t>
+          <t>32616431081</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1217,7 +1336,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Поставка спецодежды для защиты от термических рисков электрической дуги</t>
+          <t>Поставка спецодежды</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1227,33 +1346,43 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-10-15 08:00</t>
+          <t>2026-10-19 08:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>1477969</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>1108476.75</v>
-      </c>
-      <c r="I13" s="3" t="n">
+        <v>3637476.36</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Жилет сигнальный: 14 Штука × ?; Жилет утепленный: 64 Штука × ?; Костюм летний  мужской противоэнцэфалитный: 1 Комплект × ?; Костюм летний мужской для защиты от механичес: 23 Комплект × ?; Костюм летний женский для защиты от механичес: 1 Комплект × ?; Куртка зимняя мужской для защиты от механичес: 20 Штука × ?; Полукомбинезон зимний мужской для защиты от м: 20 Штука × ?; Костюм летний мужской сигнальный флуоресцентн: 4 Комплект × ?; … ещё 28</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2728107.27</v>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J13" s="3" t="n">
+      <c r="L13" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K13" s="2" t="n">
-        <v>210730.4397120549</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>210730.4397120549</v>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="2" t="n">
+        <v>518635.365684263</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>518635.365684263</v>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1267,53 +1396,61 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10749746</t>
+          <t>32616448893</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Боханский Аграрный Техникум»</t>
+          <t>Государственное автономное учреждение Московской обл. «Мособллес»</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Приобретение мягкого инвентаря, индивидуальная одежда и обувь для каждого студента. согласно спецификации и списка размеров.</t>
+          <t>Поставка обуви специальной для защиты от механических воздействий</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Малые закупки</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-10-14 10:00</t>
+          <t>2026-10-16 10:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>498000</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>373500</v>
-      </c>
-      <c r="I14" s="3" t="n">
+        <v>2511958.68</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Ботинки с высоким берцем утепленные: 396 Пара (2 шт.) × ?; Ботинки с высоким берцем утепленные: 396 Пара (2 шт.) × ? (цена за ед. = НМЦК / кол-во)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>3171.665</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1883969.01</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J14" s="3" t="n">
+      <c r="L14" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K14" s="2" t="n">
-        <v>71005.38575342466</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>71005.38575342466</v>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="2" t="n">
+        <v>358157.8214258302</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>358157.8214258302</v>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1327,53 +1464,63 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0173200001426002006</t>
+          <t>32616427138</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Московская Административная Дорожная Инспекция</t>
+          <t>Федеральное бюджетное учреждение «Государственный Региональный Центр Стандартизации, Метрологии и Испытаний Им. А.М. Муратшина в Республике Башкортостан»</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Поставка форменной одежды</t>
+          <t>Поставка спецодежды для защиты от термических рисков электрической дуги</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-10-15 10:00</t>
+          <t>2026-10-15 08:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>435666.4</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>326749.8</v>
-      </c>
-      <c r="I15" s="3" t="n">
+        <v>1477969</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Костюм летний для защиты от термических риско: 15 Комплект × ?; Костюм зимний для защиты от термических риско: 8 Комплект × ?; Куртка-рубашка для защиты от термических риск: 11 Штука × ?; Куртка-накидка для защиты от термических риск: 10 Штука × ?; Плащ термостойкий для защиты от термических р: 1 Штука × ?; Бельё нательное (фуфайка): 26 Штука × ?; Бельё нательное (кальсоны): 26 Штука × ?; Бельё нательное утепленное (фуфайка): 12 Штука × ?; … ещё 12</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>1108476.75</v>
+      </c>
+      <c r="K15" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="L15" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K15" s="2" t="n">
-        <v>62117.79275463011</v>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>62117.79275463011</v>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="2" t="n">
+        <v>210730.4397120549</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>210730.4397120549</v>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1387,17 +1534,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10747873</t>
+          <t>10749746</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Тулунский Аграрный Техникум»</t>
+          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Боханский Аграрный Техникум»</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Приобретение мягкого инвентаря Подбор индивидуальный одежды и обуви для каждого воспитанника .В случае несоответствии размера произвести замену товара, не повторяющиеся модели с учетом выбора воспитанников</t>
+          <t>Приобретение мягкого инвентаря, индивидуальная одежда и обувь для каждого студента. согласно спецификации и списка размеров.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1407,33 +1554,39 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-10-14 11:20</t>
+          <t>2026-10-14 10:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>402140</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>301605</v>
-      </c>
-      <c r="I16" s="3" t="n">
+        <v>498000</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n">
+        <v>373500</v>
+      </c>
+      <c r="K16" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J16" s="3" t="n">
+      <c r="L16" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K16" s="2" t="n">
-        <v>57337.56190136987</v>
-      </c>
-      <c r="L16" s="2" t="n">
-        <v>57337.56190136987</v>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="2" t="n">
+        <v>71005.38575342466</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>71005.38575342466</v>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1447,53 +1600,61 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10747880</t>
+          <t>0173200001426002006</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Тулунский Аграрный Техникум»</t>
+          <t>Московская Административная Дорожная Инспекция</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Приобретение мягкого инвентаря Подбор индивидуальный одежды и обуви для каждого воспитанника .В случае несоответствии размера произвести замену товара, не повторяющиеся модели с учетом выбора воспитанников</t>
+          <t>Поставка форменной одежды</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Малые закупки</t>
+          <t>44-ФЗ</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-10-14 11:20</t>
+          <t>2026-10-15 10:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>402140</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>301605</v>
-      </c>
-      <c r="I17" s="3" t="n">
+        <v>435666.4</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Термобелье спортивное, для взрослого: 2 шт × 6 100; Шорты: 2 шт × 4 266.67; Термобелье спортивное, для взрослого: 4 шт × 5 033.33; Футболка трикотажная: 2 шт × 1 033.33; Футболка трикотажная: 8 шт × 1 033.33; Шорты: 4 шт × 4 266.67; Шорты: 6 шт × 4 266.67; Шорты: 6 шт × 4 266.67; … ещё 29</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>2562.743529411765</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>326749.8</v>
+      </c>
+      <c r="K17" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J17" s="3" t="n">
+      <c r="L17" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K17" s="2" t="n">
-        <v>57337.56190136987</v>
-      </c>
-      <c r="L17" s="2" t="n">
-        <v>57337.56190136987</v>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M17" s="2" t="n">
+        <v>62117.79275463011</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>62117.79275463011</v>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1507,53 +1668,59 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0358300160926000018</t>
+          <t>10747873</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>МКУ «Управление по Делам Гражданской Обороны, Предупреждения и Ликвидации Чрезвычайных Ситуаций Города Каменск-Шахтинский»</t>
+          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Тулунский Аграрный Техникум»</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Поставка специальной одежды</t>
+          <t>Приобретение мягкого инвентаря Подбор индивидуальный одежды и обуви для каждого воспитанника .В случае несоответствии размера произвести замену товара, не повторяющиеся модели с учетом выбора воспитанников</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>Малые закупки</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-15 10:00</t>
+          <t>2026-10-14 11:20</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>320700.06</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>240525.045</v>
-      </c>
-      <c r="I18" s="3" t="n">
+        <v>402140</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n">
+        <v>301605</v>
+      </c>
+      <c r="K18" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="L18" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K18" s="2" t="n">
-        <v>45725.76600692053</v>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>45725.76600692053</v>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="M18" s="2" t="n">
+        <v>57337.56190136987</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>57337.56190136987</v>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1567,53 +1734,59 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0301300019426000247</t>
+          <t>10747880</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ГБУЗ Республиканский Клинический Госпиталь Ветеранов Войн им. М.В. Каменева</t>
+          <t>Государственное бюджетное Профессиональное Образовательное учреждение Иркутской обл. «Тулунский Аграрный Техникум»</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Поставка спецодежды</t>
+          <t>Приобретение мягкого инвентаря Подбор индивидуальный одежды и обуви для каждого воспитанника .В случае несоответствии размера произвести замену товара, не повторяющиеся модели с учетом выбора воспитанников</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>Малые закупки</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-15 07:00</t>
+          <t>2026-10-14 11:20</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>270651</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>202988.25</v>
-      </c>
-      <c r="I19" s="3" t="n">
+        <v>402140</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n">
+        <v>301605</v>
+      </c>
+      <c r="K19" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J19" s="3" t="n">
+      <c r="L19" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K19" s="2" t="n">
-        <v>38589.7161838356</v>
-      </c>
-      <c r="L19" s="2" t="n">
-        <v>38589.7161838356</v>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M19" s="2" t="n">
+        <v>57337.56190136987</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>57337.56190136987</v>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1627,17 +1800,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0302200020326000023</t>
+          <t>0358300160926000018</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Республиканская служба по охране, контролю и регулированию использования объектов животного мира, отнесенных к объектам охоты, контролю и надзору в сфере природопользования</t>
+          <t>МКУ «Управление по Делам Гражданской Обороны, Предупреждения и Ликвидации Чрезвычайных Ситуаций Города Каменск-Шахтинский»</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Поставка спецобуви</t>
+          <t>Поставка специальной одежды</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1647,33 +1820,43 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-10-14 04:00</t>
+          <t>2026-10-15 10:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>230181</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>172635.75</v>
-      </c>
-      <c r="I20" s="3" t="n">
+        <v>320700.06</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Ботинки с высокими берцами зимние: 18 пар × 5 400; Футболка поло с длинным рукавом: 18 шт × 2 800; Головной убор зимний: 18 шт × 750; Костюм спасателя мужской зимний: 18 шт × 8 866.67</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>разные позиции — см. колонку слева</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>240525.045</v>
+      </c>
+      <c r="K20" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J20" s="3" t="n">
+      <c r="L20" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K20" s="2" t="n">
-        <v>32819.45923315067</v>
-      </c>
-      <c r="L20" s="2" t="n">
-        <v>32819.45923315067</v>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M20" s="2" t="n">
+        <v>45725.76600692053</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>45725.76600692053</v>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1687,17 +1870,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0340100009726000070</t>
+          <t>0301300019426000247</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Федеральное государственное бюджетное Профессиональное Образовательное учреждение «Орловское Специальное Учебно-Воспитательное Учреждение Закрытого Типа»</t>
+          <t>ГБУЗ Республиканский Клинический Госпиталь Ветеранов Войн им. М.В. Каменева</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Поставка зимней одежды для воспитанников (термобелье)</t>
+          <t>Поставка спецодежды</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1707,33 +1890,41 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-15 08:30</t>
+          <t>2026-10-15 07:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>213567.9</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>160175.925</v>
-      </c>
-      <c r="I21" s="3" t="n">
+        <v>270651</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Костюм мужской рабочий  (96/170): 1 шт × 4 857; Костюм мужской рабочий  (104/165): 1 шт × 4 857; Костюм мужской рабочий  (104/176): 2 шт × 4 857; Костюм мужской рабочий  (108/170): 3 шт × 4 857; Костюм мужской рабочий  (108/176): 3 шт × 4 857; Костюм мужской рабочий  (112/170): 2 шт × 4 857; Костюм мужской рабочий  (112/176): 1 шт × 4 857; Костюм мужской рабочий  (96/158): 1 шт × 5 600; … ещё 29</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>5012.055555555556</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>202988.25</v>
+      </c>
+      <c r="K21" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J21" s="3" t="n">
+      <c r="L21" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K21" s="2" t="n">
-        <v>30450.74522901369</v>
-      </c>
-      <c r="L21" s="2" t="n">
-        <v>30450.74522901369</v>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M21" s="2" t="n">
+        <v>38589.7161838356</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>38589.7161838356</v>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1747,53 +1938,61 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>32616452815</t>
+          <t>0302200020326000023</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Государственное автономное учреждение Здравоохранения «Городская Больница № 2 г. Магнитогорск»</t>
+          <t>Республиканская служба по охране, контролю и регулированию использования объектов животного мира, отнесенных к объектам охоты, контролю и надзору в сфере природопользования</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Поставка комплектов зимней спецодежды и рукавиц</t>
+          <t>Поставка спецобуви</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>223-ФЗ</t>
+          <t>44-ФЗ</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-15 07:00</t>
+          <t>2026-10-14 04:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>187355.52</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>140516.64</v>
-      </c>
-      <c r="I22" s="3" t="n">
+        <v>230181</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Ботинки специальные с высокими берцами зимние: 18 пар × 3 639; Ботинки специальные с высокими берцами: 17 пар × 8 299; Обувь демисезонная: 4 пар × 5 899</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>5902.076923076923</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>172635.75</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J22" s="3" t="n">
+      <c r="L22" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K22" s="2" t="n">
-        <v>26713.3553627178</v>
-      </c>
-      <c r="L22" s="2" t="n">
-        <v>26713.3553627178</v>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M22" s="2" t="n">
+        <v>32819.45923315067</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>32819.45923315067</v>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1807,53 +2006,61 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>295997-26LO</t>
+          <t>0340100009726000070</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>МКУ «Городское Хозяйство» Муниципального Образования Волосовское Городское Поселение Волосовского Муниципального Района Ленинградской Области</t>
+          <t>Федеральное государственное бюджетное Профессиональное Образовательное учреждение «Орловское Специальное Учебно-Воспитательное Учреждение Закрытого Типа»</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Поставка товаров согласно Спецификации (Специальная одежда и обувь)</t>
+          <t>Поставка зимней одежды для воспитанников (термобелье)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Малые закупки</t>
+          <t>44-ФЗ</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-13 10:30</t>
+          <t>2026-10-15 08:30</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>152190</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>114142.5</v>
-      </c>
-      <c r="I23" s="3" t="n">
+        <v>213567.9</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Белье нательное трикотажное или вязаное: 1 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 4 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 3 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 2 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 1 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 1 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 2 КОМПЛ × 2 033.98; Белье нательное трикотажное или вязаное: 2 КОМПЛ × 2 033.98; … ещё 29</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>2033.98</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>160175.925</v>
+      </c>
+      <c r="K23" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J23" s="3" t="n">
+      <c r="L23" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K23" s="2" t="n">
-        <v>21699.41698356164</v>
-      </c>
-      <c r="L23" s="2" t="n">
-        <v>21699.41698356164</v>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="2" t="n">
+        <v>30450.74522901369</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>30450.74522901369</v>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1867,60 +2074,856 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>32616452815</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Государственное автономное учреждение Здравоохранения «Городская Больница № 2 г. Магнитогорск»</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Поставка комплектов зимней спецодежды и рукавиц</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:00</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>187355.52</v>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Костюм утепленный Ангара: 16 Комплект × ?; Рукавицы утепленные G14: 16 Пара (2 шт.) × ?</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>140516.64</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>26713.3553627178</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>26713.3553627178</v>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>Участвовать, если ≤2 заявок</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Одежда</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>295997-26LO</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>МКУ «Городское Хозяйство» Муниципального Образования Волосовское Городское Поселение Волосовского Муниципального Района Ленинградской Области</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Поставка товаров согласно Спецификации (Специальная одежда и обувь)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Малые закупки</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-10-13 10:30</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>152190</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n">
+        <v>114142.5</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>21699.41698356164</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>21699.41698356164</v>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>Участвовать, если ≤2 заявок</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Одежда</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>1022079</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Краевое ГКУ Для Детей-Сирот и Детей, Оставшихся без Попечения Родителей «Шушенский Детский Дом»</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Закупка одежды</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Коммерческие</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>2026-10-15 20:00</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>114000</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>нет данных (коммерческая/малая закупка или позиции не опубликованы)</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n">
         <v>85500</v>
       </c>
-      <c r="I24" s="3" t="n">
+      <c r="K26" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="J24" s="3" t="n">
+      <c r="L26" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="M26" s="2" t="n">
         <v>16254.24493150685</v>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="N26" s="2" t="n">
         <v>16254.24493150685</v>
       </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="O26" s="6" t="inlineStr">
         <is>
           <t>Участвовать, если ≤2 заявок</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0348300075526000435</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ГБУЗ МО «Королёвская клиническая больница» (ЦКДЛ), лот 7</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Контейнеры вакуумные для мочи</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>19.10.2026 10:00 МСК</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Контейнер вакуумный для мочи 10 мл, 15–16х100: 21 667 шт × 20.64; Контейнер вакуумный для мочи 6,5–7 мл, 13х100: 21 667 шт × 10.66; Контейнер вакуумный для мочи 9–9,5 мл, 16х100: 21 667 шт × 22.70; Контейнер вакуумный для мочи 9,5 мл, 16х100, : 21 667 шт × 15.23</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>17.30742603959939</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>1087916.66</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>0.2747222266666667</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>279266.7297835617</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>253970.7297835617</v>
+      </c>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>Осторожно</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Цены поставщика не найдены публично — себестоимость ГИПОТЕЗА (85% от цены победителя-инкумбента). Количество не определено (qty условные: НМЦК/Σцен ед. поровну). Ограничение ПП 1875: импорт (ZMT, Китай) допускается, но отклоняется при ≥2 заявках с российскими изделиями. Сильный инкумбент (выигрывает</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0387200029826000340</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>БУ ХМАО-Югры «Нижневартовская окружная клиническая больница»</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные (8 видов)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>16.10.2026 07:00 МСК</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>900000</v>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная K2ЭДТА 2–? мл 13х75, кол-в: 8 154 шт × 12.86; Пробирка вакуумная цитрат 3,8% 3–? мл 13х75, : 8 154 шт × 12.87; Пробирка вакуумная тромбин 4,5 мл 13х75, кол-: 8 154 шт × 12.10; Пробирка вакуумная K-оксалат/NaF 4,5 мл 13х75: 8 154 шт × 14.72; Пробирка вакуумная активатор 5–? мл 13х(90–10: 8 154 шт × 14.67; Пробирка вакуумная цитрат 3,8% 4–? мл 13х75, : 8 154 шт × 12.88; Пробирка вакуумная K2ЭДТА 4–? мл 13х75, кол-в: 8 154 шт × 12.87; Пробирка вакуумная Li-гепарин 4–? мл 13х75, к: 8 154 шт × 17.40</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>13.79690949227373</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>617434.5</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0.3139616666666666</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>190924.8400684932</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>1204.840068493151</v>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>Осторожно</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Количество не определено — qty условные (НМЦК/Σцен ед. поровну). Доставка в Нижневартовск (дорогая логистика). Контракт до 31.03.2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Кабель (ЭОМ)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>32616445794</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>АО «Гидроремонт-ВКК» (группа РусГидро), Саратовский филиал</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Кабель (27.32)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>15.10.2026 12:00 МСК</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>2176178.2</v>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>поз.1 ОКПД2 27.32.13.144 Кабели высоковольтны: 100 Метр × ?; поз.2 ОКПД2 27.32.13.111 Кабели силовые с мед: 300 Метр × ?; поз.3 ОКПД2 27.32.13.130 Провода и шнуры сило: 0.07 Километр; тысяча метров × ?; поз.4 ОКПД2 27.32.13.111 Кабели силовые с мед: 120 Метр × ?; поз.5 ОКПД2 27.32.13.130 Провода и шнуры сило: 50 Метр × ?; поз.6 ОКПД2 27.32.13.111 Кабели силовые с мед: 0.22 Километр; тысяча метров × ?; поз.7 ОКПД2 27.32.13.124 Кабели силовые гибки: 1.30 Километр; тысяча метров × ?; поз.8 ОКПД2 27.32.13.111 Кабели силовые с мед: 0.06 Километр; тысяча метров × ?; … ещё 10</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2" t="n"/>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>НМЦ 2 176 178,20 в ЕИС — БЕЗ НДС (rostender показывает 2 654 937 с НДС 22%). Клиент на УСН: уточнить в ДоЗ правило сравнения цен (у РусГидро обычно без НДС). Флаги нацрежима по всем 18 позициям = false (ЕИС), но ПП №1875 для 27.32 может быть указан в ДоЗ — проверить. Цены поставщиков не подобраны: н</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Кабель (ЭОМ)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>32616445272</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>АО «Гидроремонт-ВКК» (группа РусГидро), Воткинский филиал</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Кабель (27.32)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>15.10.2026 12:00 МСК</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>1201357.95</v>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>поз.1 ОКПД2 27.32.13.159 Кабели, провода и шн: 135 Метр × ?; поз.2 ОКПД2 27.32.13.131 Провода силовые для : 0.10 Километр; тысяча метров × ?; поз.3 ОКПД2 27.32.13.130 Провода и шнуры сило: 100 Метр × ?; поз.4 ОКПД2 27.32.14.111 Кабели силовые с мед: 0.06 Километр; тысяча метров × ?; поз.5 ОКПД2 27.32.13.130 Провода и шнуры сило: 60 Метр × ?; поз.6 ОКПД2 27.32.13.111 Кабели силовые с мед: 115 Метр × ?; поз.7 ОКПД2 27.32.13.111 Кабели силовые с мед: 100 Метр × ?; поз.8 ОКПД2 27.32.13.143 Кабели контрольные (: 0.20 Километр; тысяча метров × ?; … ещё 7</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>разные ед. изм.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2" t="n"/>
+      <c r="O30" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>НМЦ 1 201 357,95 без НДС (rostender: 1 465 656 с НДС). Флаги нацрежима false. Цены не подобраны — нет марок/сечений.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Кабель (ЭОМ)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>32616445510</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>АО «НИОПИК»</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Кабель (27.32)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>14.10.2026 10:00 МСК</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>529280.65</v>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Кабель сигнальный КИМЭлВ-ЗГнг(А) (ОКПД2 27.32: 1 усл. ед. × 529 280.65</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>529280.65</v>
+      </c>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="2" t="n"/>
+      <c r="N31" s="2" t="n"/>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Цена за метр не определена: неизвестны длина и конструкция. Ориентир по аналогам 1х2х0,75 (КПСнг(А)-FRHF, МКЭШВнг(А)-LS) 30–60 ₽/м с НДС — для КИМ неприменимо без спецификации. ЭТП РТС-тендер.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0855200000526003358</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Каменская ЦРБ им. Г.М. Савельевой»; организатор ГКУ ПО «Управление по осуществлению закупок Пензенской обл.»</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные (цитрат/K3/активатор)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>15.10.2026 08:00 МСК</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>1432800</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с цитратом натрия 3,8%, 4–: 15 600 шт × 10.80; Пробирка вакуумная K3ЭДТА 3–? мл 13х75 (КТРУ : 50 400 шт × 10.80; Пробирка вакуумная с активатором свертывания : 60 000 шт × 12</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>11.37142857142857</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>1171120</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0.1826353992183138</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>103594.3298630137</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>-233458.7178082192</v>
+      </c>
+      <c r="O32" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Запас НМЦК к цене МедРТ 17–20% — при медианной скидке 25% убыток; работает только с заводской ценой. Контракт до 30.12.2027 (поставка партиями — длинный оборот). СМП-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0809500000326003912</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ГБУЗ РМ «Республиканская клиническая больница им. С.В. Каткова»; организатор ГКУ РМ «Региональный центр организации закупок»</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные K3ЭДТА</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>16.10.2026 09:00 МСК</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>950000</v>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная K3ЭДТА 2–? мл 13х75, пласт: 95 000 шт × 10</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>852400</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0.1027368421052632</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>-3413.698630136991</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>-239013.698630137</v>
+      </c>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>НМЦК 10,00 ₽ vs дистрибьютор 8,92 ₽ (запас 11%) — убыточно при любой скидке &gt;11% без заводской цены. Контракт до 30.12.2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0164200001926003491</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, Тамбовская КЦРБ, онкодиспансер, Петровская, Мичуринская ЦРБ, ТОДКБ и др.)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные K3ЭДТА</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>19.10.2026 07:00 МСК</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>1691688</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с K3ЭДТА, пластик, 2–2,7 м: 35 000 шт × 9.24; То же, поз.2: 54 500 шт × 9.58; То же, поз.3: 25 000 шт × 9.93; То же, поз.4: 10 000 шт × 10.32; То же, поз.5: 2 400 шт × 10.72; То же, поз.6: 50 000 шт × 9.38</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>9.56296212549463</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>1587948</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0.06132336459205243</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>10112.2218739726</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>-407641.8923835617</v>
+      </c>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Совместная закупка (9 контрактов/адресов). Запрет иностранного. Маржа по прайсу дистрибьютора ~6% до снижения; победители по K3 в 09–10.2026 отдавали по 8.75–10.16 ₽.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0164200001926003492</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, ТОДКБ, Тамбовская КЦРБ, онкодиспансер, Петровская, Уметская, Бондарская ЦРБ и др.); организатор — уполномоченный орган Тамбовской обл.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные с активатором свёртывания</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>19.10.2026 07:00 МСК</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>2815055</v>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с активатором свертывания,: 60 000 шт × 9.89; То же, поз.2: 115 900 шт × 10.15; То же, поз.3: 20 000 шт × 10.31; То же, поз.4: 36 000 шт × 10.92; То же, поз.5: 45 000 шт × 9.91</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>10.16632358252077</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>2484948</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0.1172648491770143</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>157285.0023013699</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>-513092.4608219178</v>
+      </c>
+      <c r="O35" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Совместная закупка: 9 отдельных контрактов, 9 адресов, приёмка у каждого. Запрет иностранного (нужен РФ-производитель). Крупный лот (2.8 млн) привлечёт производителей/крупных дилеров — высокая вероятность глубокого снижения. Контракты до 25–30.12.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0335200014926003799</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Совместная закупка 26 ГБУЗ Калининградской обл.; организатор ГКУ КО «Центр обеспечения организации и проведения торгов»</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные (совместная закупка, гель/NaF)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>26.10.2026 10:00 МСК</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>5909000</v>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с активатором свертывания/: 94 122 шт × 12.29; Пробирка вакуумная с K-оксалатом и NaF 4 мл 1: 94 122 шт × 9.90; Пробирка вакуумная с активатором/гелем 5 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 6 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 5,5 мл: 94 122 шт × 13.53</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>12.55604428295191</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>5187766.56</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0.1220567676425792</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>89623.21567123328</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>-1359992.922739726</v>
+      </c>
+      <c r="O36" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Количество не определено (контракт на сумму, цена за ед.) — qty условные: НМЦК поделена поровну по позициям (НМЦК/Σцен ед.). 26 отдельных контрактов, ~26 точек доставки в эксклаве (транзит через ЛТ/паром), срок до 31.07.2027. NaF-пробирка: дистрибьюторская цена 10,93 &gt; НМЦК 9,90 — убыточна без завод</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N24"/>
+  <autoFilter ref="A1:P36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1931,7 +2934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1939,22 +2942,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Лотов</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>«Участвовать»</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Прибыль по «Участвовать», ₽</t>
         </is>
@@ -1979,16 +2982,48 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>556474.3205479452</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Кабель (ЭОМ)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>68554.01568482628</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Одежда</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B5" t="n">
         <v>20</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C5" t="n">
         <v>20</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D5" s="2" t="n">
         <v>7525368.13277052</v>
       </c>
     </row>

</xml_diff>

<commit_message>
TENDERS_1210.xlsx: add СС lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TENDERS_1210.xlsx
+++ b/TENDERS_1210.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$P$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$P$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2585,272 +2585,232 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Медрасходники</t>
+          <t>СС</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0855200000526003358</t>
+          <t>32616449701</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ГБУЗ «Каменская ЦРБ им. Г.М. Савельевой»; организатор ГКУ ПО «Управление по осуществлению закупок Пензенской обл.»</t>
+          <t>НАО «Центр «Омега» (Краснодарский край)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные (цитрат/K3/активатор)</t>
+          <t>Видеонаблюдение (СС, поставка)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>15.10.2026 08:00 МСК</t>
+          <t>16.10.2026 10:00 МСК</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>1432800</v>
+        <v>3229618.2</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Пробирка вакуумная с цитратом натрия 3,8%, 4–: 15 600 шт × 10.80; Пробирка вакуумная K3ЭДТА 3–? мл 13х75 (КТРУ : 50 400 шт × 10.80; Пробирка вакуумная с активатором свертывания : 60 000 шт × 12</t>
+          <t>Видеорегистратор (26.40.33.114): 1 шт × ?; Видеокамера тип 1 (26.40.33.111): 20 шт × ?; Видеокамера тип 2: 30 шт × ?; Видеокамера тип 3: 30 шт × ?; Видеокамера тип 4: 20 шт × ?; Аппаратура коммуникационная передающая (26.30: 1 шт × ?; Панели/комплекты электр. аппаратуры (27.12.31: 2 шт × ?; Приборы для телекоммуникаций (26.51.44, тесте: 1 шт × ?; … ещё 2 (цена за ед. = НМЦК / кол-во)</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>11.37142857142857</v>
-      </c>
-      <c r="J32" s="2" t="n">
-        <v>1171120</v>
-      </c>
-      <c r="K32" s="4" t="n">
-        <v>0.1826353992183138</v>
-      </c>
-      <c r="L32" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M32" s="2" t="n">
-        <v>103594.3298630137</v>
-      </c>
-      <c r="N32" s="2" t="n">
-        <v>-233458.7178082192</v>
-      </c>
-      <c r="O32" s="8" t="inlineStr">
-        <is>
-          <t>Нет</t>
+        <v>23923.09777777778</v>
+      </c>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Запас НМЦК к цене МедРТ 17–20% — при медианной скидке 25% убыток; работает только с заводской ценой. Контракт до 30.12.2027 (поставка партиями — длинный оборот). СМП-only.</t>
+          <t>Поставка (АЭФ только СМП), РТС-тендер Id=4056547. Монтаж в предмете не указан, но проверить проект договора. unit_nmck неизвестны → covered_nmck приравнен nmck условно, маржа по гипотезам ненадёжна. Нужна ручная выгрузка Обоснования НМЦД.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Медрасходники</t>
+          <t>СС</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0809500000326003912</t>
+          <t>32616433554</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ГБУЗ РМ «Республиканская клиническая больница им. С.В. Каткова»; организатор ГКУ РМ «Региональный центр организации закупок»</t>
+          <t>СПбГУ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные K3ЭДТА</t>
+          <t>Видеонаблюдение (СС, поставка)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>16.10.2026 09:00 МСК</t>
+          <t>14.10.2026 08:00 МСК</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>950000</v>
+        <v>1675767</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Пробирка вакуумная K3ЭДТА 2–? мл 13х75, пласт: 95 000 шт × 10</t>
+          <t>Видеокамера (26.40.33.111): 41 шт × ?; Части/принадлежности видеооборудования (кронш: 41 шт × ?; Части/принадлежности видеооборудования (короб: 41 шт × ?; Видеорегистратор: 2 шт × ?; Базовые системы хранения данных (HDD?): 16 шт × ? (цена за ед. = НМЦК / кол-во)</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J33" s="2" t="n">
-        <v>852400</v>
-      </c>
-      <c r="K33" s="4" t="n">
-        <v>0.1027368421052632</v>
-      </c>
-      <c r="L33" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M33" s="2" t="n">
-        <v>-3413.698630136991</v>
-      </c>
-      <c r="N33" s="2" t="n">
-        <v>-239013.698630137</v>
-      </c>
-      <c r="O33" s="8" t="inlineStr">
-        <is>
-          <t>Нет</t>
+        <v>11884.87234042553</v>
+      </c>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>НМЦК 10,00 ₽ vs дистрибьютор 8,92 ₽ (запас 11%) — убыточно при любой скидке &gt;11% без заводской цены. Контракт до 30.12.2027.</t>
+          <t>АЭФ только СМП, РТС-тендер Id=4052238. Поставка, монтаж не указан. unit_nmck неизвестны → covered_nmck = nmck условно.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Медрасходники</t>
+          <t>СС</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0164200001926003491</t>
+          <t>32616419880</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, Тамбовская КЦРБ, онкодиспансер, Петровская, Мичуринская ЦРБ, ТОДКБ и др.)</t>
+          <t>ФГБУ «ФЦТОЭ» Минздрава России (г. Чебоксары)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные K3ЭДТА</t>
+          <t>Видеонаблюдение (СС, поставка)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>19.10.2026 07:00 МСК</t>
+          <t>15.10.2026 14:00 МСК</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1691688</v>
+        <v>878563.71</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Пробирка вакуумная с K3ЭДТА, пластик, 2–2,7 м: 35 000 шт × 9.24; То же, поз.2: 54 500 шт × 9.58; То же, поз.3: 25 000 шт × 9.93; То же, поз.4: 10 000 шт × 10.32; То же, поз.5: 2 400 шт × 10.72; То же, поз.6: 50 000 шт × 9.38</t>
+          <t>Видеорегистратор (26.40.33.114): 1 шт × ?; Камера видеонаблюдения (26.70.13.000): 16 шт × ?; Коммутатор (26.30.11.110): 3 шт × ? (цена за ед. = НМЦК / кол-во)</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>9.56296212549463</v>
-      </c>
-      <c r="J34" s="2" t="n">
-        <v>1587948</v>
-      </c>
-      <c r="K34" s="4" t="n">
-        <v>0.06132336459205243</v>
-      </c>
-      <c r="L34" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M34" s="2" t="n">
-        <v>10112.2218739726</v>
-      </c>
-      <c r="N34" s="2" t="n">
-        <v>-407641.8923835617</v>
-      </c>
-      <c r="O34" s="8" t="inlineStr">
-        <is>
-          <t>Нет</t>
+        <v>43928.1855</v>
+      </c>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2" t="n"/>
+      <c r="O34" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Совместная закупка (9 контрактов/адресов). Запрет иностранного. Маржа по прайсу дистрибьютора ~6% до снижения; победители по K3 в 09–10.2026 отдавали по 8.75–10.16 ₽.</t>
+          <t>Документация (.docx) недоступна. unit_nmck неизвестны → covered_nmck = nmck условно.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Медрасходники</t>
+          <t>СС</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0164200001926003492</t>
+          <t>32616439096</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, ТОДКБ, Тамбовская КЦРБ, онкодиспансер, Петровская, Уметская, Бондарская ЦРБ и др.); организатор — уполномоченный орган Тамбовской обл.</t>
+          <t>СПб ГБУК «Михайловский театр»</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные с активатором свёртывания</t>
+          <t>Телеком-оборудование и расходники (СКС, низкий приоритет)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>44-ФЗ</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>19.10.2026 07:00 МСК</t>
+          <t>13.10.2026 09:00 МСК</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>2815055</v>
+        <v>987824.58</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Пробирка вакуумная с активатором свертывания,: 60 000 шт × 9.89; То же, поз.2: 115 900 шт × 10.15; То же, поз.3: 20 000 шт × 10.31; То же, поз.4: 36 000 шт × 10.92; То же, поз.5: 45 000 шт × 9.91</t>
+          <t>ITK оптический пигтейл: 240 шт/м × ?; Кабель оптический: 900 шт/м × ?; Кросс оптический: 10 шт/м × ?; Шкаф телеком. тип 1: 1 шт/м × ?; Шкаф телеком. тип 2: 2 шт/м × ?; Патч-корды типы 1–5: 160 шт/м × ?; Лоток глухой ЛМГ: 10 шт/м × ?; Кабель-канал типы 1–2: 44 шт/м × ?; … ещё 13 (цена за ед. = НМЦК / кол-во)</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>10.16632358252077</v>
-      </c>
-      <c r="J35" s="2" t="n">
-        <v>2484948</v>
-      </c>
-      <c r="K35" s="4" t="n">
-        <v>0.1172648491770143</v>
-      </c>
-      <c r="L35" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M35" s="2" t="n">
-        <v>157285.0023013699</v>
-      </c>
-      <c r="N35" s="2" t="n">
-        <v>-513092.4608219178</v>
-      </c>
-      <c r="O35" s="8" t="inlineStr">
-        <is>
-          <t>Нет</t>
+        <v>528.2484385026738</v>
+      </c>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>Нет цен — запросить КП</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Совместная закупка: 9 отдельных контрактов, 9 адресов, приёмка у каждого. Запрет иностранного (нужен РФ-производитель). Крупный лот (2.8 млн) привлечёт производителей/крупных дилеров — высокая вероятность глубокого снижения. Контракты до 25–30.12.2026.</t>
+          <t>Пропущено: низкий приоритет, срок истекает, не профиль видеонаблюдения. Себестоимость не оценивалась.</t>
         </is>
       </c>
     </row>
@@ -2862,17 +2822,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0335200014926003799</t>
+          <t>0855200000526003358</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Совместная закупка 26 ГБУЗ Калининградской обл.; организатор ГКУ КО «Центр обеспечения организации и проведения торгов»</t>
+          <t>ГБУЗ «Каменская ЦРБ им. Г.М. Савельевой»; организатор ГКУ ПО «Управление по осуществлению закупок Пензенской обл.»</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Пробирки вакуумные (совместная закупка, гель/NaF)</t>
+          <t>Пробирки вакуумные (цитрат/K3/активатор)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2882,48 +2842,390 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>26.10.2026 10:00 МСК</t>
+          <t>15.10.2026 08:00 МСК</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>5909000</v>
+        <v>1432800</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Пробирка вакуумная с активатором свертывания/: 94 122 шт × 12.29; Пробирка вакуумная с K-оксалатом и NaF 4 мл 1: 94 122 шт × 9.90; Пробирка вакуумная с активатором/гелем 5 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 6 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 5,5 мл: 94 122 шт × 13.53</t>
+          <t>Пробирка вакуумная с цитратом натрия 3,8%, 4–: 15 600 шт × 10.80; Пробирка вакуумная K3ЭДТА 3–? мл 13х75 (КТРУ : 50 400 шт × 10.80; Пробирка вакуумная с активатором свертывания : 60 000 шт × 12</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>12.55604428295191</v>
+        <v>11.37142857142857</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>5187766.56</v>
+        <v>1171120</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>0.1220567676425792</v>
+        <v>0.1826353992183138</v>
       </c>
       <c r="L36" s="4" t="n">
         <v>0.25</v>
       </c>
       <c r="M36" s="2" t="n">
+        <v>103594.3298630137</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>-233458.7178082192</v>
+      </c>
+      <c r="O36" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Запас НМЦК к цене МедРТ 17–20% — при медианной скидке 25% убыток; работает только с заводской ценой. Контракт до 30.12.2027 (поставка партиями — длинный оборот). СМП-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0809500000326003912</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ГБУЗ РМ «Республиканская клиническая больница им. С.В. Каткова»; организатор ГКУ РМ «Региональный центр организации закупок»</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные K3ЭДТА</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>16.10.2026 09:00 МСК</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>950000</v>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная K3ЭДТА 2–? мл 13х75, пласт: 95 000 шт × 10</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>852400</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0.1027368421052632</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>-3413.698630136991</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>-239013.698630137</v>
+      </c>
+      <c r="O37" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>НМЦК 10,00 ₽ vs дистрибьютор 8,92 ₽ (запас 11%) — убыточно при любой скидке &gt;11% без заводской цены. Контракт до 30.12.2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>СС</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0171100002826000003</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Управление Минюста России по Ярославской области</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Видеонаблюдение (СС, поставка)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>15.10.2026 09:00 МСК</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>588408.7</v>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Камера видеонаблюдения КТРУ 26.70.13.000-0000: 21 шт × 6 059.67; Коммутатор: 2 шт × 10 851; Трансивер: 1 шт × 2 185.67; Трансивер: 1 шт × 2 184; Источник бесперебойного питания (1): 1 шт × 15 589; Источник бесперебойного питания (2): 1 шт × 21 507; Блок розеток: 2 шт × 1 356.67; Шкаф телекоммуникационный: 2 шт × 15 799.67; … ещё 9</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>разные позиции — см. колонку слева</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>745107.8</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>-0.2663099644855695</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>-193660.3510794521</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>-336667.2015274521</v>
+      </c>
+      <c r="O38" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Запрос котировок, СМП, обеспечение исполнения 30%. Ограничение (ПП 1875) на все позиции. Камера: КТРУ требует матрицу ≤1/3" при 5 Мп 2560×1920 и НМЦК 6 060 ₽ — типичная спецификация Hikvision/HiWatch; реестровые TRASSIR 5 Мп (1/2.8") стоят от 11,3–13,4 тыс. опт и формально не подходят по размеру мат</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0164200001926003491</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, Тамбовская КЦРБ, онкодиспансер, Петровская, Мичуринская ЦРБ, ТОДКБ и др.)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные K3ЭДТА</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>19.10.2026 07:00 МСК</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>1691688</v>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с K3ЭДТА, пластик, 2–2,7 м: 35 000 шт × 9.24; То же, поз.2: 54 500 шт × 9.58; То же, поз.3: 25 000 шт × 9.93; То же, поз.4: 10 000 шт × 10.32; То же, поз.5: 2 400 шт × 10.72; То же, поз.6: 50 000 шт × 9.38</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>9.56296212549463</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>1587948</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0.06132336459205243</v>
+      </c>
+      <c r="L39" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>10112.2218739726</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>-407641.8923835617</v>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Совместная закупка (9 контрактов/адресов). Запрет иностранного. Маржа по прайсу дистрибьютора ~6% до снижения; победители по K3 в 09–10.2026 отдавали по 8.75–10.16 ₽.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0164200001926003492</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Совместная закупка 9 ТОГБУЗ Тамбовской обл. (ГКП №5, ГКБ №4, ТОДКБ, Тамбовская КЦРБ, онкодиспансер, Петровская, Уметская, Бондарская ЦРБ и др.); организатор — уполномоченный орган Тамбовской обл.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные с активатором свёртывания</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>19.10.2026 07:00 МСК</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>2815055</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с активатором свертывания,: 60 000 шт × 9.89; То же, поз.2: 115 900 шт × 10.15; То же, поз.3: 20 000 шт × 10.31; То же, поз.4: 36 000 шт × 10.92; То же, поз.5: 45 000 шт × 9.91</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>10.16632358252077</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>2484948</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0.1172648491770143</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>157285.0023013699</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>-513092.4608219178</v>
+      </c>
+      <c r="O40" s="8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Совместная закупка: 9 отдельных контрактов, 9 адресов, приёмка у каждого. Запрет иностранного (нужен РФ-производитель). Крупный лот (2.8 млн) привлечёт производителей/крупных дилеров — высокая вероятность глубокого снижения. Контракты до 25–30.12.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Медрасходники</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0335200014926003799</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Совместная закупка 26 ГБУЗ Калининградской обл.; организатор ГКУ КО «Центр обеспечения организации и проведения торгов»</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Пробирки вакуумные (совместная закупка, гель/NaF)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>26.10.2026 10:00 МСК</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>5909000</v>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Пробирка вакуумная с активатором свертывания/: 94 122 шт × 12.29; Пробирка вакуумная с K-оксалатом и NaF 4 мл 1: 94 122 шт × 9.90; Пробирка вакуумная с активатором/гелем 5 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 6 мл 1: 94 122 шт × 13.53; Пробирка вакуумная с активатором/гелем 5,5 мл: 94 122 шт × 13.53</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>12.55604428295191</v>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>5187766.56</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0.1220567676425792</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M41" s="2" t="n">
         <v>89623.21567123328</v>
       </c>
-      <c r="N36" s="2" t="n">
+      <c r="N41" s="2" t="n">
         <v>-1359992.922739726</v>
       </c>
-      <c r="O36" s="8" t="inlineStr">
+      <c r="O41" s="8" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>Количество не определено (контракт на сумму, цена за ед.) — qty условные: НМЦК поделена поровну по позициям (НМЦК/Σцен ед.). 26 отдельных контрактов, ~26 точек доставки в эксклаве (транзит через ЛТ/паром), срок до 31.07.2027. NaF-пробирка: дистрибьюторская цена 10,93 &gt; НМЦК 9,90 — убыточна без завод</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P36"/>
+  <autoFilter ref="A1:P41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2934,7 +3236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3027,6 +3329,22 @@
         <v>7525368.13277052</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>СС</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
TENDERS_1210.xlsx: flag hypothetical costs; gear and plumbing results
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TENDERS_1210.xlsx
+++ b/TENDERS_1210.xlsx
@@ -904,7 +904,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Цены по позициям в извещении не указаны: НМЦ лота задана одной суммой, документация (zip) на zakupki.gov.ru, доступа к ней нет, поэтому unit_nmck не указаны. У Т Плюс НМЦ часто указана без НДС — проверить; для УСН это важно. Около половины позиций (энергетические вентили ВТ-5, ВИГ, 15с27нж, 14с17п, </t>
+          <t xml:space="preserve">[ГИПОТЕЗА по себестоимости] Цены по позициям в извещении не указаны: НМЦ лота задана одной суммой, документация (zip) на zakupki.gov.ru, доступа к ней нет, поэтому unit_nmck не указаны. У Т Плюс НМЦ часто указана без НДС — проверить; для УСН это важно. Около половины позиций (энергетические вентили ВТ-5, ВИГ, 15с27нж, 14с17п, </t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Цены по позициям не указаны в извещении; длины плеч, диаметр оболочки и наличие проводников ОДК — в документах (недоступны). Тяжёлый груз (426/530 — по 200–300 кг), доставка в Уфу — оценка 45 тыс. Уфимские производители ППУ (например, местные заводы) имеют логистическое преимущество. Не СМП-закупка.</t>
+          <t>[ГИПОТЕЗА по себестоимости] Цены по позициям не указаны в извещении; длины плеч, диаметр оболочки и наличие проводников ОДК — в документах (недоступны). Тяжёлый груз (426/530 — по 200–300 кг), доставка в Уфу — оценка 45 тыс. Уфимские производители ППУ (например, местные заводы) имеют логистическое преимущество. Не СМП-закупка.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Сечения и доля КНРЭ неизвестны — себестоимость гипотетична. Розничные цены агрегаторов (Рукабель, kabel-s) 170–440 ₽/м выше средней НМЦК 260,6 ₽/м → если в лоте 3х2,5 и крупнее, маржи может не быть; реально только при цене завода (Кольчугино/Рыбинсккабель/Камкабель) ~126–154 ₽/м за 3х2,5 и малых сеч</t>
+          <t>[ГИПОТЕЗА по себестоимости] Сечения и доля КНРЭ неизвестны — себестоимость гипотетична. Розничные цены агрегаторов (Рукабель, kabel-s) 170–440 ₽/м выше средней НМЦК 260,6 ₽/м → если в лоте 3х2,5 и крупнее, маржи может не быть; реально только при цене завода (Кольчугино/Рыбинсккабель/Камкабель) ~126–154 ₽/м за 3х2,5 и малых сеч</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Цены поставщика не найдены публично — себестоимость ГИПОТЕЗА (85% от цены победителя-инкумбента). Количество не определено (qty условные: НМЦК/Σцен ед. поровну). Ограничение ПП 1875: импорт (ZMT, Китай) допускается, но отклоняется при ≥2 заявках с российскими изделиями. Сильный инкумбент (выигрывает</t>
+          <t>[ГИПОТЕЗА по себестоимости] Цены поставщика не найдены публично — себестоимость ГИПОТЕЗА (85% от цены победителя-инкумбента). Количество не определено (qty условные: НМЦК/Σцен ед. поровну). Ограничение ПП 1875: импорт (ZMT, Китай) допускается, но отклоняется при ≥2 заявках с российскими изделиями. Сильный инкумбент (выигрывает</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Диаметры и типы неизвестны: ТЗ в rar на zakupki.gov.ru, доступа нет. Запрос котировок для МСП на ЭТП РАД (lot-online). Флаг нацрежима стоит → нужен российский производитель. Малый лот, логистика съедает маржу.</t>
+          <t>[ГИПОТЕЗА по себестоимости] Диаметры и типы неизвестны: ТЗ в rar на zakupki.gov.ru, доступа нет. Запрос котировок для МСП на ЭТП РАД (lot-online). Флаг нацрежима стоит → нужен российский производитель. Малый лот, логистика съедает маржу.</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Приём заявок заканчивается завтра (13.10.2026 05:00 МСК) — успеть практически нереально. Запрет ПП 1875: нужна реестровая запись российского производителя. Цена — гипотеза.</t>
+          <t>[ГИПОТЕЗА по себестоимости] Приём заявок заканчивается завтра (13.10.2026 05:00 МСК) — успеть практически нереально. Запрет ПП 1875: нужна реестровая запись российского производителя. Цена — гипотеза.</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Ограничение ПП 1875 (кроме фланцев — преимущество): нужна арматура российского производства с номером реестровой записи РПП (Челарм, СибЗТА — проверить реестр). ТЗ: задвижки чугунные PN16 металл-по-металлу — 30ч6бр это Ру10; под PN16 нужна 30ч515бр/30ч15бр (цена по запросу, вероятно дороже). Затворы</t>
+          <t>[ГИПОТЕЗА по себестоимости] Ограничение ПП 1875 (кроме фланцев — преимущество): нужна арматура российского производства с номером реестровой записи РПП (Челарм, СибЗТА — проверить реестр). ТЗ: задвижки чугунные PN16 металл-по-металлу — 30ч6бр это Ру10; под PN16 нужна 30ч515бр/30ч15бр (цена по запросу, вероятно дороже). Затворы</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Срок подачи 15.10 09:00 МСК — осталось меньше 3 дней. ТЗ и обоснование НМЦД (xls) лежат на zakupki.gov.ru, доступа к ним нет: характеристики (ткань, плотность, наполнитель, размеры) и цены по позициям неизвестны, поэтому вся себестоимость — гипотеза. Вероятна высокая конкуренция ивановских производи</t>
+          <t>[ГИПОТЕЗА по себестоимости] Срок подачи 15.10 09:00 МСК — осталось меньше 3 дней. ТЗ и обоснование НМЦД (xls) лежат на zakupki.gov.ru, доступа к ним нет: характеристики (ткань, плотность, наполнитель, размеры) и цены по позициям неизвестны, поэтому вся себестоимость — гипотеза. Вероятна высокая конкуренция ивановских производи</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Запрос котировок, СМП, обеспечение исполнения 30%. Ограничение (ПП 1875) на все позиции. Камера: КТРУ требует матрицу ≤1/3" при 5 Мп 2560×1920 и НМЦК 6 060 ₽ — типичная спецификация Hikvision/HiWatch; реестровые TRASSIR 5 Мп (1/2.8") стоят от 11,3–13,4 тыс. опт и формально не подходят по размеру мат</t>
+          <t>[ГИПОТЕЗА по себестоимости] Запрос котировок, СМП, обеспечение исполнения 30%. Ограничение (ПП 1875) на все позиции. Камера: КТРУ требует матрицу ≤1/3" при 5 Мп 2560×1920 и НМЦК 6 060 ₽ — типичная спецификация Hikvision/HiWatch; реестровые TRASSIR 5 Мп (1/2.8") стоят от 11,3–13,4 тыс. опт и формально не подходят по размеру мат</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TENDERS_1210.xlsx: add advance, bid and contract security, SMP, ETP columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TENDERS_1210.xlsx
+++ b/TENDERS_1210.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Коммерческие без НМЦК" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$P$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Тендеры 12.10'!$A$1:$U$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Коммерческие без НМЦК'!$A$1:$H$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:U48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -483,7 +483,12 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="60" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +569,31 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Аванс</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Обеспечение заявки</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Обеспечение исполнения контракта</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Только СМП</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Площадка (ЭТП)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Комментарий</t>
         </is>
       </c>
@@ -632,6 +662,31 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>ЭТП ГПБ</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
           <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ на эквивалент</t>
         </is>
       </c>
@@ -700,6 +755,27 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>67 240 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>672 400 ₽ (10.0%)</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
           <t>223-ФЗ; обеспечение исполнения 10%</t>
         </is>
       </c>
@@ -768,6 +844,31 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ</t>
         </is>
       </c>
@@ -836,6 +937,31 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>14 760 ₽ (0.5%)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>5.00 % (≈147 600 ₽)</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Росэлторг (ЕЭТП)</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
           <t>НМЦК 19,68 ₽ — вдвое выше рынка, поэтому ожидается сильное снижение (вероятно верхний квартиль скидки, 40–55%). Особенность крышки (полнозаходная резьба / двухступенчатое снятие) — нужно подтвердить, что UNIVAC/другая российская пробирка этому соответствует, иначе отклонение. СМП-only. Минимальный о</t>
         </is>
       </c>
@@ -904,6 +1030,27 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>ПАО «Т‑Плюс»</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
           <t xml:space="preserve">[ГИПОТЕЗА по себестоимости] Цены по позициям в извещении не указаны: НМЦ лота задана одной суммой, документация (zip) на zakupki.gov.ru, доступа к ней нет, поэтому unit_nmck не указаны. У Т Плюс НМЦ часто указана без НДС — проверить; для УСН это важно. Около половины позиций (энергетические вентили ВТ-5, ВИГ, 15с27нж, 14с17п, </t>
         </is>
       </c>
@@ -972,6 +1119,27 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Российская электронная система торгов</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Цены по позициям не указаны в извещении; длины плеч, диаметр оболочки и наличие проводников ОДК — в документах (недоступны). Тяжёлый груз (426/530 — по 200–300 кг), доставка в Уфу — оценка 45 тыс. Уфимские производители ППУ (например, местные заводы) имеют логистическое преимущество. Не СМП-закупка.</t>
         </is>
       </c>
@@ -1040,6 +1208,31 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>есть, размер в документации</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>ЭТП ГПБ</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Сечения и доля КНРЭ неизвестны — себестоимость гипотетична. Розничные цены агрегаторов (Рукабель, kabel-s) 170–440 ₽/м выше средней НМЦК 260,6 ₽/м → если в лоте 3х2,5 и крупнее, маржи может не быть; реально только при цене завода (Кольчугино/Рыбинсккабель/Камкабель) ~126–154 ₽/м за 3х2,5 и малых сеч</t>
         </is>
       </c>
@@ -1110,6 +1303,31 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>180 339 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>10.00 % (≈1 803 387 ₽)</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1180,6 +1398,31 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>62 244 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>10.00 % (≈622 442 ₽)</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1248,6 +1491,31 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Центр Закупок Республики Саха (Якутия)</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1315,6 +1583,31 @@
         </is>
       </c>
       <c r="P12" t="inlineStr">
+        <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1382,6 +1675,27 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>ЭТП ГПБ</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1452,6 +1766,31 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1522,6 +1861,27 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1590,6 +1950,31 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>125 598 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1659,6 +2044,27 @@
         </is>
       </c>
       <c r="P17" t="inlineStr">
+        <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1726,6 +2132,31 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1793,6 +2224,31 @@
         </is>
       </c>
       <c r="P19" t="inlineStr">
+        <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>4 357 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>5.00 % (≈21 783 ₽)</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Росэлторг (ЕЭТП)</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -1860,6 +2316,27 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1926,6 +2403,27 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -1996,6 +2494,31 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>5.00 % (≈16 035 ₽)</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2064,6 +2587,27 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1 353 ₽ (0.5%)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>27 065 ₽ (10.0%)</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2132,6 +2676,31 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1.00 % (≈2 302 ₽)</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2200,6 +2769,31 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2 136 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>10.00 % (≈21 357 ₽)</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Росэлторг (ЕЭТП)</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2269,6 +2863,31 @@
         </is>
       </c>
       <c r="P26" t="inlineStr">
+        <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Информационная система "Управление закупками отдельными видами юридических лиц"</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
         <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
@@ -2336,6 +2955,27 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Электронный Магазин Ленинградской области</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2402,6 +3042,27 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>ЭТП ГПБ</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
           <t>себестоимость = 75% НМЦК (данные клиента), снижение ≤5%</t>
         </is>
       </c>
@@ -2470,6 +3131,27 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>15 000 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>150 000 ₽ (10.0%)</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Росэлторг (ЕЭТП)</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Цены поставщика не найдены публично — себестоимость ГИПОТЕЗА (85% от цены победителя-инкумбента). Количество не определено (qty условные: НМЦК/Σцен ед. поровну). Ограничение ПП 1875: импорт (ZMT, Китай) допускается, но отклоняется при ≥2 заявках с российскими изделиями. Сильный инкумбент (выигрывает</t>
         </is>
       </c>
@@ -2538,6 +3220,31 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>РАД (Lot-Online)</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Диаметры и типы неизвестны: ТЗ в rar на zakupki.gov.ru, доступа нет. Запрос котировок для МСП на ЭТП РАД (lot-online). Флаг нацрежима стоит → нужен российский производитель. Малый лот, логистика съедает маржу.</t>
         </is>
       </c>
@@ -2605,6 +3312,27 @@
         </is>
       </c>
       <c r="P31" t="inlineStr">
+        <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>90 000 ₽ (10.0%)</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
         <is>
           <t>Количество не определено — qty условные (НМЦК/Σцен ед. поровну). Доставка в Нижневартовск (дорогая логистика). Контракт до 31.03.2027.</t>
         </is>
@@ -2666,6 +3394,27 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
+          <t>есть, размер в документации</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>РАД (Lot-Online)</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
           <t>НМЦ 2 176 178,20 в ЕИС — БЕЗ НДС (rostender показывает 2 654 937 с НДС 22%). Клиент на УСН: уточнить в ДоЗ правило сравнения цен (у РусГидро обычно без НДС). Флаги нацрежима по всем 18 позициям = false (ЕИС), но ПП №1875 для 27.32 может быть указан в ДоЗ — проверить. Цены поставщиков не подобраны: н</t>
         </is>
       </c>
@@ -2726,6 +3475,27 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
+          <t>есть, размер в документации</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>РАД (Lot-Online)</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
           <t>НМЦ 1 201 357,95 без НДС (rostender: 1 465 656 с НДС). Флаги нацрежима false. Цены не подобраны — нет марок/сечений.</t>
         </is>
       </c>
@@ -2784,6 +3554,31 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
+          <t>есть, размер в документации</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
           <t>Цена за метр не определена: неизвестны длина и конструкция. Ориентир по аналогам 1х2х0,75 (КПСнг(А)-FRHF, МКЭШВнг(А)-LS) 30–60 ₽/м с НДС — для КИМ неприменимо без спецификации. ЭТП РТС-тендер.</t>
         </is>
       </c>
@@ -2842,6 +3637,31 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>161 481 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
           <t>Поставка (АЭФ только СМП), РТС-тендер Id=4056547. Монтаж в предмете не указан, но проверить проект договора. unit_nmck неизвестны → covered_nmck приравнен nmck условно, маржа по гипотезам ненадёжна. Нужна ручная выгрузка Обоснования НМЦД.</t>
         </is>
       </c>
@@ -2900,6 +3720,31 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>83 788 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
           <t>АЭФ только СМП, РТС-тендер Id=4052238. Поставка, монтаж не указан. unit_nmck неизвестны → covered_nmck = nmck условно.</t>
         </is>
       </c>
@@ -2958,6 +3803,27 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>87 856 ₽ (10.0%)</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
           <t>Документация (.docx) недоступна. unit_nmck неизвестны → covered_nmck = nmck условно.</t>
         </is>
       </c>
@@ -3016,6 +3882,31 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>49 391 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
           <t>Пропущено: низкий приоритет, срок истекает, не профиль видеонаблюдения. Себестоимость не оценивалась.</t>
         </is>
       </c>
@@ -3084,6 +3975,31 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1.00 % (≈1 900 ₽)</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Приём заявок заканчивается завтра (13.10.2026 05:00 МСК) — успеть практически нереально. Запрет ПП 1875: нужна реестровая запись российского производителя. Цена — гипотеза.</t>
         </is>
       </c>
@@ -3152,6 +4068,31 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>5.00 % (≈26 298 ₽)</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Ограничение ПП 1875 (кроме фланцев — преимущество): нужна арматура российского производства с номером реестровой записи РПП (Челарм, СибЗТА — проверить реестр). ТЗ: задвижки чугунные PN16 металл-по-металлу — 30ч6бр это Ру10; под PN16 нужна 30ч515бр/30ч15бр (цена по запросу, вероятно дороже). Затворы</t>
         </is>
       </c>
@@ -3220,6 +4161,31 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
           <t>НМЦК за комплект 105 100 ₽ против розницы производителя 107 500 ₽ (УП-5 68 000 + ПБ-1 28 500 + соединитель 11 000) — маржа будет только при дилерской скидке Берега (обычно 15–25% для перепродавцов; нужно запросить). Цены по позициям в извещении не указаны, разбивка unit_nmck — оценка пропорционально</t>
         </is>
       </c>
@@ -3290,6 +4256,31 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Срок подачи 15.10 09:00 МСК — осталось меньше 3 дней. ТЗ и обоснование НМЦД (xls) лежат на zakupki.gov.ru, доступа к ним нет: характеристики (ткань, плотность, наполнитель, размеры) и цены по позициям неизвестны, поэтому вся себестоимость — гипотеза. Вероятна высокая конкуренция ивановских производи</t>
         </is>
       </c>
@@ -3358,6 +4349,31 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>14 328 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>5.00 % (≈71 640 ₽)</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
           <t>Запас НМЦК к цене МедРТ 17–20% — при медианной скидке 25% убыток; работает только с заводской ценой. Контракт до 30.12.2027 (поставка партиями — длинный оборот). СМП-only.</t>
         </is>
       </c>
@@ -3426,6 +4442,31 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>не установлено / не указано</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>5.00 % (≈47 500 ₽)</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>РАД (Lot-Online)</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
           <t>НМЦК 10,00 ₽ vs дистрибьютор 8,92 ₽ (запас 11%) — убыточно при любой скидке &gt;11% без заводской цены. Контракт до 30.12.2027.</t>
         </is>
       </c>
@@ -3496,6 +4537,31 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>5 884 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>30.00 % (≈176 523 ₽)</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Для СМП, СОНО</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Сбербанк-АСТ</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
           <t>[ГИПОТЕЗА по себестоимости] Запрос котировок, СМП, обеспечение исполнения 30%. Ограничение (ПП 1875) на все позиции. Камера: КТРУ требует матрицу ≤1/3" при 5 Мп 2560×1920 и НМЦК 6 060 ₽ — типичная спецификация Hikvision/HiWatch; реестровые TRASSIR 5 Мп (1/2.8") стоят от 11,3–13,4 тыс. опт и формально не подходят по размеру мат</t>
         </is>
       </c>
@@ -3564,6 +4630,27 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>16 917 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>84 584 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>ЭТП «Фабрикант»</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
           <t>Совместная закупка (9 контрактов/адресов). Запрет иностранного. Маржа по прайсу дистрибьютора ~6% до снижения; победители по K3 в 09–10.2026 отдавали по 8.75–10.16 ₽.</t>
         </is>
       </c>
@@ -3632,6 +4719,27 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>28 151 ₽ (1.0%)</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>140 753 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>ЭТП «Фабрикант»</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
           <t>Совместная закупка: 9 отдельных контрактов, 9 адресов, приёмка у каждого. Запрет иностранного (нужен РФ-производитель). Крупный лот (2.8 млн) привлечёт производителей/крупных дилеров — высокая вероятность глубокого снижения. Контракты до 25–30.12.2026.</t>
         </is>
       </c>
@@ -3700,12 +4808,33 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
+          <t>нет / не указан</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>7 500 ₽ (0.1%)</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>295 450 ₽ (5.0%)</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
           <t>Количество не определено (контракт на сумму, цена за ед.) — qty условные: НМЦК поделена поровну по позициям (НМЦК/Σцен ед.). 26 отдельных контрактов, ~26 точек доставки в эксклаве (транзит через ЛТ/паром), срок до 31.07.2027. NaF-пробирка: дистрибьюторская цена 10,93 &gt; НМЦК 9,90 — убыточна без завод</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P48"/>
+  <autoFilter ref="A1:U48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix salt profit columns in TENDERS_1210.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/TENDERS_1210.xlsx
+++ b/TENDERS_1210.xlsx
@@ -647,10 +647,10 @@
         <v>0.8291182501708817</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>9262976.735973697</v>
+        <v>9613813.031013699</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>7859631.555813699</v>
@@ -687,7 +687,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ на эквивалент</t>
+          <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ на эквивалент; снижение 15% — консервативно (медиана по соли 3%)</t>
         </is>
       </c>
     </row>
@@ -740,10 +740,10 @@
         <v>0.851279000594884</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>4621641.290520548</v>
+        <v>4791731.594520547</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>3941280.074520547</v>
@@ -776,7 +776,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>223-ФЗ; обеспечение исполнения 10%</t>
+          <t>223-ФЗ; обеспечение исполнения 10%; снижение 15% — консервативно (медиана по соли 3%)</t>
         </is>
       </c>
     </row>
@@ -922,10 +922,10 @@
         <v>0.7960848287112561</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1018243.203419178</v>
+        <v>1058559.968219178</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>856976.144219178</v>
@@ -962,7 +962,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ</t>
+          <t>223-ФЗ; «Концентрат минеральный Галит» — сверить ТЗ; снижение 15% — консервативно (медиана по соли 3%)</t>
         </is>
       </c>
     </row>

</xml_diff>